<commit_message>
Refactored stage 1, added HZD toxicity mty method, Updated MRT with Python modules.
</commit_message>
<xml_diff>
--- a/results/02_taxa_assemblage/MRT_Method/classifier_prediction/artifacts/mrt_predicted_data.xlsx
+++ b/results/02_taxa_assemblage/MRT_Method/classifier_prediction/artifacts/mrt_predicted_data.xlsx
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -559,7 +559,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
         <v>1</v>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
         <v>1</v>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" t="n">
         <v>1</v>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
         <v>1</v>
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C31" t="n">
         <v>1</v>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C33" t="n">
         <v>1</v>
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C34" t="n">
         <v>1</v>
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35" t="n">
         <v>0</v>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C36" t="n">
         <v>0</v>
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" t="n">
         <v>1</v>
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" t="n">
         <v>0</v>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C41" t="n">
         <v>0</v>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C42" t="n">
         <v>0</v>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C44" t="n">
         <v>0</v>
@@ -1014,7 +1014,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C45" t="n">
         <v>0</v>
@@ -1027,10 +1027,10 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C47" t="n">
         <v>1</v>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" t="n">
         <v>1</v>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C51" t="n">
         <v>1</v>
@@ -1131,7 +1131,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C54" t="n">
         <v>1</v>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C57" t="n">
         <v>1</v>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C58" t="n">
         <v>0</v>
@@ -1196,7 +1196,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C59" t="n">
         <v>1</v>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C64" t="n">
         <v>1</v>
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C66" t="n">
         <v>0</v>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C69" t="n">
         <v>0</v>
@@ -1378,7 +1378,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C73" t="n">
         <v>0</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C75" t="n">
         <v>0</v>
@@ -1430,7 +1430,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C77" t="n">
         <v>0</v>
@@ -1443,7 +1443,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C78" t="n">
         <v>0</v>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C87" t="n">
         <v>0</v>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C88" t="n">
         <v>0</v>
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C94" t="n">
         <v>1</v>
@@ -1664,7 +1664,7 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C95" t="n">
         <v>1</v>
@@ -1693,7 +1693,7 @@
         <v>2</v>
       </c>
       <c r="C97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C99" t="n">
         <v>0</v>
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C100" t="n">
         <v>1</v>
@@ -1768,7 +1768,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C103" t="n">
         <v>1</v>
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C104" t="n">
         <v>1</v>
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C105" t="n">
         <v>0</v>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C106" t="n">
         <v>0</v>
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C107" t="n">
         <v>1</v>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C109" t="n">
         <v>0</v>
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C110" t="n">
         <v>0</v>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C111" t="n">
         <v>0</v>
@@ -1911,7 +1911,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C114" t="n">
         <v>0</v>
@@ -1924,7 +1924,7 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C115" t="n">
         <v>1</v>
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C116" t="n">
         <v>0</v>
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C117" t="n">
         <v>0</v>
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C118" t="n">
         <v>0</v>
@@ -1976,7 +1976,7 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C119" t="n">
         <v>0</v>
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C121" t="n">
         <v>1</v>
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C122" t="n">
         <v>0</v>
@@ -2028,7 +2028,7 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C123" t="n">
         <v>1</v>
@@ -2054,7 +2054,7 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C125" t="n">
         <v>0</v>
@@ -2080,7 +2080,7 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C127" t="n">
         <v>0</v>
@@ -2093,7 +2093,7 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C128" t="n">
         <v>1</v>
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C132" t="n">
         <v>1</v>
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C135" t="n">
         <v>0</v>
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C136" t="n">
         <v>0</v>
@@ -2210,7 +2210,7 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C137" t="n">
         <v>0</v>
@@ -2236,7 +2236,7 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C139" t="n">
         <v>0</v>
@@ -2249,7 +2249,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C140" t="n">
         <v>0</v>
@@ -2275,7 +2275,7 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C142" t="n">
         <v>0</v>
@@ -2288,7 +2288,7 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C143" t="n">
         <v>0</v>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C145" t="n">
         <v>0</v>
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C146" t="n">
         <v>0</v>
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="B150" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C150" t="n">
         <v>0</v>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="B151" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C151" t="n">
         <v>0</v>
@@ -2418,7 +2418,7 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C153" t="n">
         <v>0</v>
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="B154" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C154" t="n">
         <v>0</v>
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C156" t="n">
         <v>0</v>
@@ -2470,7 +2470,7 @@
         </is>
       </c>
       <c r="B157" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C157" t="n">
         <v>0</v>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="B160" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C160" t="n">
         <v>0</v>
@@ -2522,7 +2522,7 @@
         </is>
       </c>
       <c r="B161" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C161" t="n">
         <v>0</v>
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="B162" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C162" t="n">
         <v>0</v>
@@ -2564,7 +2564,7 @@
         <v>2</v>
       </c>
       <c r="C164" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165">
@@ -2574,7 +2574,7 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C165" t="n">
         <v>0</v>
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="B166" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C166" t="n">
         <v>0</v>
@@ -2600,7 +2600,7 @@
         </is>
       </c>
       <c r="B167" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C167" t="n">
         <v>1</v>
@@ -2626,7 +2626,7 @@
         </is>
       </c>
       <c r="B169" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C169" t="n">
         <v>1</v>
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="B170" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C170" t="n">
         <v>0</v>
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C172" t="n">
         <v>1</v>
@@ -2691,7 +2691,7 @@
         </is>
       </c>
       <c r="B174" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C174" t="n">
         <v>0</v>
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="B180" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C180" t="n">
         <v>0</v>
@@ -2782,7 +2782,7 @@
         </is>
       </c>
       <c r="B181" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C181" t="n">
         <v>0</v>
@@ -2821,7 +2821,7 @@
         </is>
       </c>
       <c r="B184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C184" t="n">
         <v>0</v>
@@ -2834,7 +2834,7 @@
         </is>
       </c>
       <c r="B185" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C185" t="n">
         <v>0</v>
@@ -2860,7 +2860,7 @@
         </is>
       </c>
       <c r="B187" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C187" t="n">
         <v>0</v>
@@ -2886,7 +2886,7 @@
         </is>
       </c>
       <c r="B189" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C189" t="n">
         <v>0</v>
@@ -2915,7 +2915,7 @@
         <v>3</v>
       </c>
       <c r="C191" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="192">
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="B192" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C192" t="n">
         <v>1</v>
@@ -2951,7 +2951,7 @@
         </is>
       </c>
       <c r="B194" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C194" t="n">
         <v>1</v>
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="B196" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C196" t="n">
         <v>0</v>
@@ -3003,7 +3003,7 @@
         </is>
       </c>
       <c r="B198" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C198" t="n">
         <v>0</v>
@@ -3016,7 +3016,7 @@
         </is>
       </c>
       <c r="B199" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C199" t="n">
         <v>0</v>
@@ -3029,7 +3029,7 @@
         </is>
       </c>
       <c r="B200" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C200" t="n">
         <v>0</v>
@@ -3042,7 +3042,7 @@
         </is>
       </c>
       <c r="B201" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C201" t="n">
         <v>0</v>
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="B202" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C202" t="n">
         <v>0</v>
@@ -3068,7 +3068,7 @@
         </is>
       </c>
       <c r="B203" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C203" t="n">
         <v>0</v>
@@ -3107,7 +3107,7 @@
         </is>
       </c>
       <c r="B206" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C206" t="n">
         <v>1</v>
@@ -3133,7 +3133,7 @@
         </is>
       </c>
       <c r="B208" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C208" t="n">
         <v>0</v>
@@ -3162,7 +3162,7 @@
         <v>3</v>
       </c>
       <c r="C210" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="211">
@@ -3172,7 +3172,7 @@
         </is>
       </c>
       <c r="B211" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C211" t="n">
         <v>1</v>
@@ -3198,7 +3198,7 @@
         </is>
       </c>
       <c r="B213" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C213" t="n">
         <v>0</v>
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="B214" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C214" t="n">
         <v>0</v>
@@ -3263,7 +3263,7 @@
         </is>
       </c>
       <c r="B218" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C218" t="n">
         <v>1</v>
@@ -3276,7 +3276,7 @@
         </is>
       </c>
       <c r="B219" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C219" t="n">
         <v>0</v>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="B220" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C220" t="n">
         <v>0</v>
@@ -3302,7 +3302,7 @@
         </is>
       </c>
       <c r="B221" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C221" t="n">
         <v>0</v>
@@ -3328,7 +3328,7 @@
         </is>
       </c>
       <c r="B223" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C223" t="n">
         <v>0</v>
@@ -3341,7 +3341,7 @@
         </is>
       </c>
       <c r="B224" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C224" t="n">
         <v>0</v>
@@ -3354,7 +3354,7 @@
         </is>
       </c>
       <c r="B225" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C225" t="n">
         <v>0</v>
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="B226" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C226" t="n">
         <v>0</v>
@@ -3380,7 +3380,7 @@
         </is>
       </c>
       <c r="B227" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C227" t="n">
         <v>0</v>
@@ -3393,7 +3393,7 @@
         </is>
       </c>
       <c r="B228" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C228" t="n">
         <v>0</v>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="B229" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C229" t="n">
         <v>0</v>
@@ -3419,7 +3419,7 @@
         </is>
       </c>
       <c r="B230" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C230" t="n">
         <v>0</v>
@@ -3432,7 +3432,7 @@
         </is>
       </c>
       <c r="B231" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C231" t="n">
         <v>0</v>
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="B233" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C233" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Added env-ordination visualization for clusters.
</commit_message>
<xml_diff>
--- a/results/02_taxa_assemblage/MRT_Method/classifier_prediction/artifacts/mrt_predicted_data.xlsx
+++ b/results/02_taxa_assemblage/MRT_Method/classifier_prediction/artifacts/mrt_predicted_data.xlsx
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -559,7 +559,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" t="n">
         <v>1</v>
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
         <v>1</v>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
@@ -676,10 +676,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -689,10 +689,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
@@ -754,10 +754,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26" t="n">
         <v>1</v>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C29" t="n">
         <v>1</v>
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C33" t="n">
         <v>1</v>
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C35" t="n">
         <v>0</v>
@@ -910,10 +910,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
@@ -936,7 +936,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C39" t="n">
         <v>0</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" t="n">
         <v>0</v>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41" t="n">
         <v>0</v>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C42" t="n">
         <v>0</v>
@@ -1014,7 +1014,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C45" t="n">
         <v>0</v>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C46" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C47" t="n">
         <v>1</v>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C48" t="n">
         <v>0</v>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C49" t="n">
         <v>1</v>
@@ -1092,10 +1092,10 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C57" t="n">
         <v>1</v>
@@ -1196,7 +1196,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C59" t="n">
         <v>1</v>
@@ -1222,7 +1222,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" t="n">
         <v>0</v>
@@ -1251,7 +1251,7 @@
         <v>1</v>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -1264,7 +1264,7 @@
         <v>1</v>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C68" t="n">
         <v>0</v>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C69" t="n">
         <v>0</v>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C70" t="n">
         <v>0</v>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C71" t="n">
         <v>0</v>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C72" t="n">
         <v>0</v>
@@ -1378,7 +1378,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C73" t="n">
         <v>0</v>
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C74" t="n">
         <v>0</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C75" t="n">
         <v>0</v>
@@ -1430,7 +1430,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C77" t="n">
         <v>0</v>
@@ -1443,7 +1443,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C78" t="n">
         <v>0</v>
@@ -1456,10 +1456,10 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C80" t="n">
         <v>0</v>
@@ -1482,7 +1482,7 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C81" t="n">
         <v>0</v>
@@ -1498,7 +1498,7 @@
         <v>3</v>
       </c>
       <c r="C82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -1508,10 +1508,10 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C84" t="n">
         <v>0</v>
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C85" t="n">
         <v>0</v>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C87" t="n">
         <v>0</v>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C88" t="n">
         <v>0</v>
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C90" t="n">
         <v>0</v>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C91" t="n">
         <v>0</v>
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C92" t="n">
         <v>0</v>
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C94" t="n">
         <v>1</v>
@@ -1664,10 +1664,10 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C98" t="n">
         <v>0</v>
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C99" t="n">
         <v>0</v>
@@ -1729,10 +1729,10 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C102" t="n">
         <v>0</v>
@@ -1768,7 +1768,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C103" t="n">
         <v>1</v>
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C104" t="n">
         <v>1</v>
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C107" t="n">
         <v>1</v>
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C110" t="n">
         <v>0</v>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C111" t="n">
         <v>0</v>
@@ -1911,7 +1911,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C114" t="n">
         <v>0</v>
@@ -1924,7 +1924,7 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C115" t="n">
         <v>1</v>
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C116" t="n">
         <v>0</v>
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C117" t="n">
         <v>0</v>
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C121" t="n">
         <v>1</v>
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C122" t="n">
         <v>0</v>
@@ -2028,10 +2028,10 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124">
@@ -2041,7 +2041,7 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C124" t="n">
         <v>0</v>
@@ -2054,7 +2054,7 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C125" t="n">
         <v>0</v>
@@ -2080,7 +2080,7 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C127" t="n">
         <v>0</v>
@@ -2093,10 +2093,10 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C128" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129">
@@ -2145,10 +2145,10 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C132" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133">
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C135" t="n">
         <v>0</v>
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C136" t="n">
         <v>0</v>
@@ -2210,7 +2210,7 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C137" t="n">
         <v>0</v>
@@ -2236,7 +2236,7 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C139" t="n">
         <v>0</v>
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C141" t="n">
         <v>0</v>
@@ -2275,7 +2275,7 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C142" t="n">
         <v>0</v>
@@ -2288,7 +2288,7 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C143" t="n">
         <v>0</v>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C145" t="n">
         <v>0</v>
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C146" t="n">
         <v>0</v>
@@ -2366,10 +2366,10 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C149" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150">
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="B150" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C150" t="n">
         <v>0</v>
@@ -2392,7 +2392,7 @@
         </is>
       </c>
       <c r="B151" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C151" t="n">
         <v>0</v>
@@ -2418,7 +2418,7 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C153" t="n">
         <v>0</v>
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="B154" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C154" t="n">
         <v>0</v>
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C156" t="n">
         <v>0</v>
@@ -2496,7 +2496,7 @@
         </is>
       </c>
       <c r="B159" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C159" t="n">
         <v>0</v>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="B160" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C160" t="n">
         <v>0</v>
@@ -2522,7 +2522,7 @@
         </is>
       </c>
       <c r="B161" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C161" t="n">
         <v>0</v>
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="B162" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C162" t="n">
         <v>0</v>
@@ -2548,7 +2548,7 @@
         </is>
       </c>
       <c r="B163" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C163" t="n">
         <v>0</v>
@@ -2564,7 +2564,7 @@
         <v>2</v>
       </c>
       <c r="C164" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165">
@@ -2574,7 +2574,7 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C165" t="n">
         <v>0</v>
@@ -2587,10 +2587,10 @@
         </is>
       </c>
       <c r="B166" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C166" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
@@ -2600,7 +2600,7 @@
         </is>
       </c>
       <c r="B167" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C167" t="n">
         <v>1</v>
@@ -2613,7 +2613,7 @@
         </is>
       </c>
       <c r="B168" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C168" t="n">
         <v>0</v>
@@ -2626,7 +2626,7 @@
         </is>
       </c>
       <c r="B169" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C169" t="n">
         <v>1</v>
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="B170" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C170" t="n">
         <v>0</v>
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C172" t="n">
         <v>1</v>
@@ -2691,7 +2691,7 @@
         </is>
       </c>
       <c r="B174" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C174" t="n">
         <v>0</v>
@@ -2756,7 +2756,7 @@
         </is>
       </c>
       <c r="B179" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C179" t="n">
         <v>0</v>
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="B180" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C180" t="n">
         <v>0</v>
@@ -2782,7 +2782,7 @@
         </is>
       </c>
       <c r="B181" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C181" t="n">
         <v>0</v>
@@ -2808,7 +2808,7 @@
         </is>
       </c>
       <c r="B183" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C183" t="n">
         <v>0</v>
@@ -2821,7 +2821,7 @@
         </is>
       </c>
       <c r="B184" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C184" t="n">
         <v>0</v>
@@ -2860,7 +2860,7 @@
         </is>
       </c>
       <c r="B187" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C187" t="n">
         <v>0</v>
@@ -2873,7 +2873,7 @@
         </is>
       </c>
       <c r="B188" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C188" t="n">
         <v>0</v>
@@ -2886,7 +2886,7 @@
         </is>
       </c>
       <c r="B189" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C189" t="n">
         <v>0</v>
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="B190" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C190" t="n">
         <v>0</v>
@@ -2915,7 +2915,7 @@
         <v>3</v>
       </c>
       <c r="C191" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192">
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="B192" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C192" t="n">
         <v>1</v>
@@ -2938,7 +2938,7 @@
         </is>
       </c>
       <c r="B193" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C193" t="n">
         <v>1</v>
@@ -2951,7 +2951,7 @@
         </is>
       </c>
       <c r="B194" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C194" t="n">
         <v>1</v>
@@ -2964,7 +2964,7 @@
         </is>
       </c>
       <c r="B195" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C195" t="n">
         <v>1</v>
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="B196" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C196" t="n">
         <v>0</v>
@@ -3029,7 +3029,7 @@
         </is>
       </c>
       <c r="B200" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C200" t="n">
         <v>0</v>
@@ -3068,7 +3068,7 @@
         </is>
       </c>
       <c r="B203" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C203" t="n">
         <v>0</v>
@@ -3081,7 +3081,7 @@
         </is>
       </c>
       <c r="B204" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C204" t="n">
         <v>0</v>
@@ -3094,7 +3094,7 @@
         </is>
       </c>
       <c r="B205" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C205" t="n">
         <v>0</v>
@@ -3107,7 +3107,7 @@
         </is>
       </c>
       <c r="B206" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C206" t="n">
         <v>1</v>
@@ -3159,10 +3159,10 @@
         </is>
       </c>
       <c r="B210" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C210" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="211">
@@ -3185,7 +3185,7 @@
         </is>
       </c>
       <c r="B212" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C212" t="n">
         <v>1</v>
@@ -3201,7 +3201,7 @@
         <v>2</v>
       </c>
       <c r="C213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="214">
@@ -3237,10 +3237,10 @@
         </is>
       </c>
       <c r="B216" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217">
@@ -3276,7 +3276,7 @@
         </is>
       </c>
       <c r="B219" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C219" t="n">
         <v>0</v>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="B220" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C220" t="n">
         <v>0</v>
@@ -3302,7 +3302,7 @@
         </is>
       </c>
       <c r="B221" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C221" t="n">
         <v>0</v>
@@ -3328,7 +3328,7 @@
         </is>
       </c>
       <c r="B223" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C223" t="n">
         <v>0</v>
@@ -3341,7 +3341,7 @@
         </is>
       </c>
       <c r="B224" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C224" t="n">
         <v>0</v>
@@ -3367,7 +3367,7 @@
         </is>
       </c>
       <c r="B226" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C226" t="n">
         <v>0</v>
@@ -3380,7 +3380,7 @@
         </is>
       </c>
       <c r="B227" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C227" t="n">
         <v>0</v>
@@ -3393,7 +3393,7 @@
         </is>
       </c>
       <c r="B228" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C228" t="n">
         <v>0</v>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="B229" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C229" t="n">
         <v>0</v>
@@ -3432,7 +3432,7 @@
         </is>
       </c>
       <c r="B231" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C231" t="n">
         <v>0</v>
@@ -3497,7 +3497,7 @@
         </is>
       </c>
       <c r="B236" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C236" t="n">
         <v>0</v>

</xml_diff>